<commit_message>
News template: tags-empty guard; docs/report updates
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-news-v1.report.xlsx
+++ b/tools/importer/reports/import-news-v1.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="880" uniqueCount="475">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="890" uniqueCount="480">
   <si>
     <t>_reportFile</t>
   </si>
@@ -1092,6 +1092,21 @@
   </si>
   <si>
     <t>https://www.ustafoundation.com/en/home/news/usta-foundation-celebrates-2026-njtl-essay-contest-winners-at-us.html</t>
+  </si>
+  <si>
+    <t>en/home/news/usta-foundation-celebrates-24-outstanding-students-through-caree.report.json</t>
+  </si>
+  <si>
+    <t>en/home/news/usta-foundation-celebrates-24-outstanding-students-through-caree</t>
+  </si>
+  <si>
+    <t>2026-09-22T09:25:54.407Z</t>
+  </si>
+  <si>
+    <t>USTA Foundation celebrates 24 outstanding students through Career Excellence Week and AMEX Excellence Cup</t>
+  </si>
+  <si>
+    <t>https://www.ustafoundation.com/en/home/news/usta-foundation-celebrates-24-outstanding-students-through-caree.html</t>
   </si>
   <si>
     <t>en/home/news/usta-foundation-chairperson-chris-evert-announces-cancer-free.report.json</t>
@@ -1828,7 +1843,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J88"/>
+  <dimension ref="A1:J89"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="5" width="50" customWidth="1"/>
@@ -3954,7 +3969,7 @@
         <v>359</v>
       </c>
       <c r="B67" t="s">
-        <v>103</v>
+        <v>79</v>
       </c>
       <c r="C67" t="s">
         <v>12</v>
@@ -4018,7 +4033,7 @@
         <v>369</v>
       </c>
       <c r="B69" t="s">
-        <v>109</v>
+        <v>103</v>
       </c>
       <c r="C69" t="s">
         <v>12</v>
@@ -4050,39 +4065,39 @@
         <v>374</v>
       </c>
       <c r="B70" t="s">
+        <v>109</v>
+      </c>
+      <c r="C70" t="s">
+        <v>12</v>
+      </c>
+      <c r="D70" t="s">
+        <v>12</v>
+      </c>
+      <c r="E70" t="s">
         <v>375</v>
       </c>
-      <c r="C70" t="s">
-        <v>12</v>
-      </c>
-      <c r="D70" t="s">
-        <v>12</v>
-      </c>
-      <c r="E70" t="s">
+      <c r="F70" t="s">
+        <v>14</v>
+      </c>
+      <c r="G70" t="s">
+        <v>74</v>
+      </c>
+      <c r="H70" t="s">
         <v>376</v>
       </c>
-      <c r="F70" t="s">
-        <v>14</v>
-      </c>
-      <c r="G70" t="s">
-        <v>74</v>
-      </c>
-      <c r="H70" t="s">
+      <c r="I70" t="s">
         <v>377</v>
       </c>
-      <c r="I70" t="s">
+      <c r="J70" t="s">
         <v>378</v>
-      </c>
-      <c r="J70" t="s">
-        <v>379</v>
       </c>
     </row>
     <row r="71" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
+        <v>379</v>
+      </c>
+      <c r="B71" t="s">
         <v>380</v>
-      </c>
-      <c r="B71" t="s">
-        <v>232</v>
       </c>
       <c r="C71" t="s">
         <v>12</v>
@@ -4114,7 +4129,7 @@
         <v>385</v>
       </c>
       <c r="B72" t="s">
-        <v>79</v>
+        <v>232</v>
       </c>
       <c r="C72" t="s">
         <v>12</v>
@@ -4178,7 +4193,7 @@
         <v>395</v>
       </c>
       <c r="B74" t="s">
-        <v>308</v>
+        <v>79</v>
       </c>
       <c r="C74" t="s">
         <v>12</v>
@@ -4210,7 +4225,7 @@
         <v>400</v>
       </c>
       <c r="B75" t="s">
-        <v>109</v>
+        <v>308</v>
       </c>
       <c r="C75" t="s">
         <v>12</v>
@@ -4274,7 +4289,7 @@
         <v>410</v>
       </c>
       <c r="B77" t="s">
-        <v>79</v>
+        <v>109</v>
       </c>
       <c r="C77" t="s">
         <v>12</v>
@@ -4338,7 +4353,7 @@
         <v>420</v>
       </c>
       <c r="B79" t="s">
-        <v>232</v>
+        <v>79</v>
       </c>
       <c r="C79" t="s">
         <v>12</v>
@@ -4370,7 +4385,7 @@
         <v>425</v>
       </c>
       <c r="B80" t="s">
-        <v>109</v>
+        <v>232</v>
       </c>
       <c r="C80" t="s">
         <v>12</v>
@@ -4402,7 +4417,7 @@
         <v>430</v>
       </c>
       <c r="B81" t="s">
-        <v>232</v>
+        <v>109</v>
       </c>
       <c r="C81" t="s">
         <v>12</v>
@@ -4466,7 +4481,7 @@
         <v>440</v>
       </c>
       <c r="B83" t="s">
-        <v>130</v>
+        <v>232</v>
       </c>
       <c r="C83" t="s">
         <v>12</v>
@@ -4498,7 +4513,7 @@
         <v>445</v>
       </c>
       <c r="B84" t="s">
-        <v>85</v>
+        <v>130</v>
       </c>
       <c r="C84" t="s">
         <v>12</v>
@@ -4530,48 +4545,48 @@
         <v>450</v>
       </c>
       <c r="B85" t="s">
+        <v>85</v>
+      </c>
+      <c r="C85" t="s">
+        <v>12</v>
+      </c>
+      <c r="D85" t="s">
+        <v>12</v>
+      </c>
+      <c r="E85" t="s">
         <v>451</v>
       </c>
-      <c r="C85" t="s">
-        <v>12</v>
-      </c>
-      <c r="D85" t="s">
-        <v>12</v>
-      </c>
-      <c r="E85" t="s">
+      <c r="F85" t="s">
+        <v>14</v>
+      </c>
+      <c r="G85" t="s">
+        <v>74</v>
+      </c>
+      <c r="H85" t="s">
         <v>452</v>
       </c>
-      <c r="F85" t="s">
-        <v>14</v>
-      </c>
-      <c r="G85" t="s">
-        <v>22</v>
-      </c>
-      <c r="H85" t="s">
+      <c r="I85" t="s">
         <v>453</v>
       </c>
-      <c r="I85" t="s">
+      <c r="J85" t="s">
         <v>454</v>
-      </c>
-      <c r="J85" t="s">
-        <v>455</v>
       </c>
     </row>
     <row r="86" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
+        <v>455</v>
+      </c>
+      <c r="B86" t="s">
         <v>456</v>
       </c>
-      <c r="B86" t="s">
+      <c r="C86" t="s">
+        <v>12</v>
+      </c>
+      <c r="D86" t="s">
+        <v>12</v>
+      </c>
+      <c r="E86" t="s">
         <v>457</v>
-      </c>
-      <c r="C86" t="s">
-        <v>12</v>
-      </c>
-      <c r="D86" t="s">
-        <v>12</v>
-      </c>
-      <c r="E86" t="s">
-        <v>458</v>
       </c>
       <c r="F86" t="s">
         <v>14</v>
@@ -4580,77 +4595,109 @@
         <v>22</v>
       </c>
       <c r="H86" t="s">
+        <v>458</v>
+      </c>
+      <c r="I86" t="s">
         <v>459</v>
       </c>
-      <c r="I86" t="s">
+      <c r="J86" t="s">
         <v>460</v>
-      </c>
-      <c r="J86" t="s">
-        <v>461</v>
       </c>
     </row>
     <row r="87" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
+        <v>461</v>
+      </c>
+      <c r="B87" t="s">
         <v>462</v>
       </c>
-      <c r="B87" t="s">
+      <c r="C87" t="s">
+        <v>12</v>
+      </c>
+      <c r="D87" t="s">
+        <v>12</v>
+      </c>
+      <c r="E87" t="s">
         <v>463</v>
       </c>
-      <c r="C87" t="s">
-        <v>12</v>
-      </c>
-      <c r="D87" t="s">
-        <v>12</v>
-      </c>
-      <c r="E87" t="s">
+      <c r="F87" t="s">
+        <v>14</v>
+      </c>
+      <c r="G87" t="s">
+        <v>22</v>
+      </c>
+      <c r="H87" t="s">
         <v>464</v>
       </c>
-      <c r="F87" t="s">
-        <v>14</v>
-      </c>
-      <c r="G87" t="s">
+      <c r="I87" t="s">
         <v>465</v>
       </c>
-      <c r="H87" t="s">
+      <c r="J87" t="s">
         <v>466</v>
-      </c>
-      <c r="I87" t="s">
-        <v>467</v>
-      </c>
-      <c r="J87" t="s">
-        <v>468</v>
       </c>
     </row>
     <row r="88" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
+        <v>467</v>
+      </c>
+      <c r="B88" t="s">
+        <v>468</v>
+      </c>
+      <c r="C88" t="s">
+        <v>12</v>
+      </c>
+      <c r="D88" t="s">
+        <v>12</v>
+      </c>
+      <c r="E88" t="s">
         <v>469</v>
       </c>
-      <c r="B88" t="s">
+      <c r="F88" t="s">
+        <v>14</v>
+      </c>
+      <c r="G88" t="s">
         <v>470</v>
       </c>
-      <c r="C88" t="s">
-        <v>12</v>
-      </c>
-      <c r="D88" t="s">
-        <v>12</v>
-      </c>
-      <c r="E88" t="s">
+      <c r="H88" t="s">
         <v>471</v>
       </c>
-      <c r="F88" t="s">
-        <v>14</v>
-      </c>
-      <c r="G88" t="s">
+      <c r="I88" t="s">
+        <v>472</v>
+      </c>
+      <c r="J88" t="s">
+        <v>473</v>
+      </c>
+    </row>
+    <row r="89" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>474</v>
+      </c>
+      <c r="B89" t="s">
+        <v>475</v>
+      </c>
+      <c r="C89" t="s">
+        <v>12</v>
+      </c>
+      <c r="D89" t="s">
+        <v>12</v>
+      </c>
+      <c r="E89" t="s">
+        <v>476</v>
+      </c>
+      <c r="F89" t="s">
+        <v>14</v>
+      </c>
+      <c r="G89" t="s">
         <v>22</v>
       </c>
-      <c r="H88" t="s">
-        <v>472</v>
-      </c>
-      <c r="I88" t="s">
-        <v>473</v>
-      </c>
-      <c r="J88" t="s">
-        <v>474</v>
+      <c r="H89" t="s">
+        <v>477</v>
+      </c>
+      <c r="I89" t="s">
+        <v>478</v>
+      </c>
+      <c r="J89" t="s">
+        <v>479</v>
       </c>
     </row>
   </sheetData>

</xml_diff>